<commit_message>
Format x-axis periods as MM/YY in RD-per-bin chart
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M73LqayoX4sQQSkWfbL6JX
</commit_message>
<xml_diff>
--- a/RD_por_bin.xlsx
+++ b/RD_por_bin.xlsx
@@ -832,8 +832,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>202309</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>09/23</t>
+        </is>
       </c>
       <c r="B2" s="1" t="n">
         <v>0.04178273</v>
@@ -855,8 +857,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>202310</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10/23</t>
+        </is>
       </c>
       <c r="B3" s="1" t="n">
         <v>0.06006006</v>
@@ -878,8 +882,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>202311</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>11/23</t>
+        </is>
       </c>
       <c r="B4" s="1" t="n">
         <v>0.06</v>
@@ -901,8 +907,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>202312</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>12/23</t>
+        </is>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.054151625</v>
@@ -924,8 +932,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>202401</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>01/24</t>
+        </is>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.058441558</v>
@@ -947,8 +957,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>202402</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>02/24</t>
+        </is>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.074433657</v>
@@ -970,8 +982,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>202403</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>03/24</t>
+        </is>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.041420118</v>
@@ -993,8 +1007,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>202404</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>04/24</t>
+        </is>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.04</v>
@@ -1016,8 +1032,10 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>202405</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>05/24</t>
+        </is>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.077306733</v>
@@ -1039,8 +1057,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>202406</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06/24</t>
+        </is>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.066489362</v>
@@ -1062,8 +1082,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>202407</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07/24</t>
+        </is>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.08114558500000001</v>
@@ -1085,8 +1107,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>202408</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08/24</t>
+        </is>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.036414566</v>
@@ -1108,8 +1132,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>202409</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>09/24</t>
+        </is>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.062645012</v>
@@ -1131,8 +1157,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>202410</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10/24</t>
+        </is>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.054545455</v>
@@ -1154,8 +1182,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>202411</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>11/24</t>
+        </is>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.051094891</v>
@@ -1177,8 +1207,10 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
-        <v>202412</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>12/24</t>
+        </is>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.08761329299999999</v>
@@ -1200,8 +1232,10 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
-        <v>202501</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>01/25</t>
+        </is>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.082644628</v>
@@ -1223,8 +1257,10 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>202502</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>02/25</t>
+        </is>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.07967033</v>

</xml_diff>